<commit_message>
feat: complete genuine 100-video evaluation results, tables, and plots
</commit_message>
<xml_diff>
--- a/evaluation/reports/evaluation_results.xlsx
+++ b/evaluation/reports/evaluation_results.xlsx
@@ -8099,17 +8099,42 @@
       </c>
       <c r="H74" s="4" t="inlineStr">
         <is>
-          <t>Error: HTTPConnectionPool(host='localhost', port=11434): Read timed out. (read timeout=180)</t>
-        </is>
-      </c>
-      <c r="I74" s="6" t="inlineStr">
-        <is>
-          <t>Low</t>
+          <t>Okay, let’s analyze this surveillance video sequence based on the provided activity class: “A man is standing outside a house, appearing to be looking into a window.”
+**1. What is happening?**
+The primary action visible in the video is a man standing outdoors and intently observing a window of a residential property. He appears to be focused on what’s inside the house. 
+**2. Which activities are visible?**
+*   **Observation:** The most prominent activity is the man's deliberate observation of the window.
+*   **Standing/Presence:**  The man is simply present outside the residence.
+*   **Movement (Minor):** He appears to be subtly adjusting his position or posture while looking at the window. 
+**3. Is there any suspicious behaviour?**
+Yes, there is potentially suspicious behavior. The fact that a person is standing outside and focused on someone else's window raises concerns. It’s not inherently suspicious, but it warrants further investigation to determine the reason for this observation.
+**4. Are there any threat indicators?**
+*   **Unidentified Individual:** We don't know who this man is or his intentions.
+*   **Privacy Violation:**  Looking into a window constitutes a potential privacy violation. 
+*   **Potential Surveillance:** The action could be part of an attempt to gather information about the occupants of the house.
+**5. Estimate the threat level as Low, Medium, or High.**
+**Threat Level: Medium**
+**6. Explain your reasoning:**
+Here’s why I assess the threat level as medium:
+*   **Uncertain Intentions:** The core issue is the unknown motivation behind the man's actions. He could be a neighbor simply curious about something, but he could also be engaged in illicit activity (e.g., stalking, reconnaissance).
+*   **Privacy Concern:**  The act of looking into a window inherently raises privacy concerns and can be unsettling for the occupants of the house. 
+*   **Lack of Immediate Danger:** There's no immediate physical threat visible in the frame – no weapons or aggressive behavior. However, the situation has the potential to escalate if the man’s intentions are not benign.
+**Recommendations:**
+*   **Monitor Further:** This video segment should be part of a larger surveillance review.
+*   **Identify the Individual:** Attempt to identify the man in the video (e.g., through facial recognition, neighborhood inquiries). 
+*   **Alert Occupants:**  The residents of the house should be notified and advised to take precautions. They might want to check their security systems or contact local law enforcement.
+---
+Would you like me to analyze a different aspect of this video, such as specific details within the frame (e.g., time of day, surrounding environment) or consider additional factors that could influence the threat assessment?</t>
+        </is>
+      </c>
+      <c r="I74" s="5" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
       <c r="J74" s="3" t="inlineStr">
         <is>
-          <t>Base: 0.00s | FT Guided: 180.06s</t>
+          <t>Base: 0.00s | FT Guided: 109.70s</t>
         </is>
       </c>
       <c r="K74" s="4" t="inlineStr">
@@ -8136,7 +8161,7 @@
       </c>
       <c r="D75" s="4" t="inlineStr">
         <is>
-          <t>Error: HTTPConnectionPool(host='localhost', port=11434): Read timed out. (read timeout=60)</t>
+          <t>Error: HTTPConnectionPool(host='localhost', port=11434): Read timed out. (read timeout=180)</t>
         </is>
       </c>
       <c r="E75" s="4" t="inlineStr">
@@ -8158,17 +8183,42 @@
       </c>
       <c r="H75" s="4" t="inlineStr">
         <is>
-          <t>Error: HTTPConnectionPool(host='localhost', port=11434): Read timed out. (read timeout=60)</t>
-        </is>
-      </c>
-      <c r="I75" s="6" t="inlineStr">
-        <is>
-          <t>Low</t>
+          <t>Okay, let’s analyze this surveillance scene video based on the provided activity class and visual evidence.
+**What is happening?**
+The image shows a residential street with two vehicles – a dark-colored sedan and a red car – parked along the curb. It appears to be a quiet suburban scene captured by a security camera. The timestamp indicates it’s a recording from October 26, 2014, at approximately 1:32:42 AM.
+**Which activities are visible?**
+*   **Vehicle Parking:** The primary activity is the presence of two vehicles parked on the street.
+*   **Street Observation:** A person (likely a resident) is visible walking along the sidewalk in the background.
+*   **Security Camera Operation:** The image itself is a recording from a security camera, indicating surveillance is taking place.
+**Is there any suspicious behaviour?**
+Based solely on this single frame, it's difficult to definitively determine if there’s *suspicious* behavior. However, several factors warrant further investigation:
+*   **Unusual Time:** The time of the recording (1:32 AM) is outside typical residential activity hours. This alone isn't necessarily suspicious but raises a flag for potential observation.
+*   **Vehicle Presence:** The parked sedan could be legitimate (e.g., someone visiting a neighbor), or it could be related to something else.
+**Are there any threat indicators?**
+There are no immediately obvious *threat indicators* in this single frame. There's no visible confrontation, violence, or anything that screams danger. However, the unusual time and the parked vehicle create an environment where further observation is needed. 
+**Estimate the threat level as Low, Medium, or High.**
+**Threat Level: Low**
+**Reasoning:**
+The image presents a low threat level based on the limited information available. Here’s my breakdown of why:
+*   **Lack of Immediate Threat:** There's no visible evidence of criminal activity in this single frame.
+*   **Context is Key:** The time of day and the parked vehicle are the primary concerns, but they don't automatically indicate a threat. It could be a normal situation.
+*   **Need for Further Investigation:** This image alone isn’t enough to make a definitive assessment.  A full review of the video footage would be necessary to determine if there is any suspicious activity or potential risk.
+**Recommendations (Based on this single frame):**
+1.  **Review Full Footage:** The most important step is to examine the entire video recording, not just this one frame.
+2.  **Identify Vehicle Owners:** Determine who owns the dark-colored sedan and the red car.
+3.  **Monitor Activity:** Observe the surrounding area for any unusual activity or individuals approaching the property.
+---
+Would you like me to analyze additional frames from the video sequence, or would you like me to elaborate on a specific aspect of this analysis?</t>
+        </is>
+      </c>
+      <c r="I75" s="5" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
       <c r="J75" s="3" t="inlineStr">
         <is>
-          <t>Base: 60.03s | FT Guided: 60.03s</t>
+          <t>Base: 180.04s | FT Guided: 104.68s</t>
         </is>
       </c>
       <c r="K75" s="4" t="inlineStr">
@@ -8219,17 +8269,41 @@
       </c>
       <c r="H76" s="4" t="inlineStr">
         <is>
-          <t>Error: HTTPConnectionPool(host='localhost', port=11434): Read timed out. (read timeout=60)</t>
-        </is>
-      </c>
-      <c r="I76" s="6" t="inlineStr">
-        <is>
-          <t>Low</t>
+          <t>Okay, based on the provided activity class ("A person is attempting to break into a building by forcefully pushing against a glass door") and the visual evidence in the image, here’s an analysis:
+**What is happening?**
+The video shows a single individual actively trying to gain unauthorized entry into a building. They are positioned directly in front of a glass-paneled door, using considerable force to push it open. 
+**Which activities are visible?**
+* **Forcible Entry Attempt:** The primary activity is the deliberate and forceful attempt to breach the security of the building.
+* **Movement:** The individual is actively moving towards the door, demonstrating intent.
+* **Physical Action:**  The pushing motion clearly indicates an effort to overcome the resistance of the door.
+**Is there any suspicious behaviour?**
+Yes, absolutely. The behavior is highly suspicious due to several factors:
+* **Targeting a Secure Area:** Approaching and attempting to force entry into a building represents a direct violation of security protocols.
+* **Forceful Action:** Using force against property suggests an intent to bypass legitimate access methods. 
+**Are there any threat indicators?**
+Yes, the image contains several threat indicators:
+* **Potential for Damage:** The forceful pushing could result in damage to the glass door and potentially other building components.
+* **Risk of Injury:**  The individual attempting this action poses a risk of injury to themselves if they are unsuccessful or if someone attempts to intervene. 
+* **Criminal Intent:** This activity strongly suggests criminal intent – burglary, vandalism, or possibly something more serious depending on the context.
+**Estimate the threat level as Low, Medium, or High.**
+I would rate the threat level as **Medium**.
+**Reasoning:**
+Here’s why I've assessed it as medium:
+* **Not Imminent Danger (Currently):** The individual hasn't yet succeeded in breaking into the building. There isn't an immediate, active threat to people or property *at this precise moment*.
+* **Significant Potential for Harm:** However, the action is clearly intended to cause damage and could easily escalate if the person gains entry.  The potential for injury (to themselves or others) remains a concern. 
+* **Criminal Activity:** The act itself constitutes criminal behavior, which carries inherent risk and potential consequences.
+**Important Note:** This assessment is based solely on this single frame of video. A full analysis would require reviewing the entire sequence to understand the individual's motivations, whether they were deterred, and any other relevant contextual information. 
+Do you want me to elaborate on a specific aspect of this analysis (e.g., potential consequences, factors influencing threat level)?</t>
+        </is>
+      </c>
+      <c r="I76" s="5" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
       <c r="J76" s="3" t="inlineStr">
         <is>
-          <t>Base: 0.00s | FT Guided: 60.01s</t>
+          <t>Base: 0.00s | FT Guided: 99.73s</t>
         </is>
       </c>
       <c r="K76" s="4" t="inlineStr">
@@ -8278,17 +8352,39 @@
       </c>
       <c r="H77" s="4" t="inlineStr">
         <is>
-          <t>Error: HTTPConnectionPool(host='localhost', port=11434): Read timed out. (read timeout=60)</t>
-        </is>
-      </c>
-      <c r="I77" s="6" t="inlineStr">
-        <is>
-          <t>Low</t>
+          <t>Okay, let's analyze this surveillance scene based on the provided activity class and visual information.
+**What is happening?**
+The video shows a young boy running across a grassy lawn towards a small, dark-colored pool. The boy appears to be in motion, actively moving across the space. 
+**Which activities are visible?**
+*   **Running:** The primary activity is the boy’s movement – he is running.
+*   **Movement Across Lawn:** He's traversing a grassy area.
+*   **Approach to Pool:**  He is heading towards a small pool.
+**Is there any suspicious behaviour?**
+Yes, there is potentially suspicious behavior. The fact that a young boy is running toward an unsupervised pool without apparent adult supervision raises concerns. While it doesn’t automatically indicate danger, it warrants closer observation. 
+**Are there any threat indicators?**
+*   **Unsupervised Pool:** Pools can be dangerous, especially for children. Without an adult present to supervise and ensure safety, the risk of accidental drowning or injury is elevated.
+*   **Lack of Adult Supervision:** The most significant indicator is the absence of a visible adult figure in the scene. This increases the potential risk significantly.
+**Estimate the threat level as Low, Medium, or High.**
+I would rate the threat level as **Medium**. 
+**Explanation of Reasoning:**
+Here’s why I've assigned a medium threat level:
+*   **Potential for Harm:** The primary concern is the unsupervised pool and the potential for an accident (drowning, slip/fall). Children can be unpredictable.
+*   **Lack of Context:** We don't know *why* the boy is running towards the pool. Is he playing? Is he lost or disoriented? Without more information, we must assume a level of risk. 
+*   **Absence of Supervision:** The lack of an adult present is the most critical factor driving this assessment. It significantly increases the potential for negative outcomes.
+**Recommendations (based on this analysis):**
+*   **Further Observation:** This scene should be monitored closely to determine the boy's intentions and whether an adult arrives to supervise.
+*   **Alert Authorities:** Depending on the duration of the event, the context, and any other observed factors, it might be prudent to alert local authorities (police or child protective services) for a precautionary check-in. 
+**Disclaimer:** *This analysis is based solely on the provided image and activity class description. A full investigation would require more detailed information about the surrounding environment, the boy's background, and any other relevant factors.*</t>
+        </is>
+      </c>
+      <c r="I77" s="5" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
       <c r="J77" s="3" t="inlineStr">
         <is>
-          <t>Base: 0.00s | FT Guided: 60.01s</t>
+          <t>Base: 0.00s | FT Guided: 97.10s</t>
         </is>
       </c>
       <c r="K77" s="4" t="inlineStr">
@@ -8337,17 +8433,44 @@
       </c>
       <c r="H78" s="4" t="inlineStr">
         <is>
-          <t>Error: HTTPConnectionPool(host='localhost', port=11434): Read timed out. (read timeout=60)</t>
-        </is>
-      </c>
-      <c r="I78" s="6" t="inlineStr">
-        <is>
-          <t>Low</t>
+          <t>Okay, let’s analyze this surveillance scene based on the provided activity class and visual evidence.
+**What is happening?**
+The primary event is a large, dark cube falling from an open doorway onto the concrete sidewalk below. The video clearly shows the object in motion and its impact with the ground. 
+**Which activities are visible?**
+* **Object Fall:** The most prominent activity is the downward trajectory of the cube.
+* **Doorway Openness:** An open doorway is present, acting as the source of the falling object.
+* **Sidewalk Presence:** A concrete sidewalk exists where the object impacts. 
+* **Reflection:** There's a reflection in the glass of the door frame, suggesting a potential camera presence and recording this event.
+**Is there any suspicious behaviour?**
+Yes, there is potentially suspicious behavior. The fact that a large cube is falling from an open doorway without apparent cause raises immediate concerns. It’s not immediately obvious *how* the cube got into the doorway or why it was released. 
+**Are there any threat indicators?**
+Absolutely. This situation presents several threat indicators:
+* **Unexplained Object:** The presence of a large, dark cube in an open doorway is unusual and warrants investigation. It could be a tool used for damage, a distraction, or part of a larger operation.
+* **Potential for Injury:**  The falling object poses a risk of injury to anyone nearby – pedestrians, staff, or customers. 
+* **Possible Malicious Intent:** The action itself suggests potential malicious intent, whether it's vandalism, an attempt to disrupt operations, or something more serious.
+**Estimate the threat level as Low, Medium, or High.**
+I would rate this threat level as **Medium**. 
+**Explain your reasoning:**
+Here’s why I assess the threat level as medium:
+*   **Uncertainty is Key:** The most significant factor is the *lack of context*. We don't know how the cube got there, who put it there, or what their intentions are. This uncertainty elevates the risk.
+*   **Potential for Harm:** While a falling object isn’t inherently catastrophic, it *can* cause damage and injury. 
+*   **Suspicious Circumstances:** The unusual nature of the event – a large cube falling from an open doorway – is highly suspicious and suggests something beyond a simple accident.
+**Recommendations:**
+1.  **Immediate Investigation:** This scene requires immediate investigation by security personnel or law enforcement.
+2.  **Secure the Area:** Establish a perimeter around the affected area to prevent further incidents and potential harm.
+3.  **Review Surveillance Footage:** Thoroughly examine all available surveillance footage from surrounding cameras to identify the origin of the cube, any individuals involved, and their movements. 
+4.  **Assess Damage:** Evaluate the damage caused by the falling object and take steps to mitigate any risks.
+Do you want me to elaborate on a specific aspect of this analysis or consider alternative threat level assessments?</t>
+        </is>
+      </c>
+      <c r="I78" s="5" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
       <c r="J78" s="3" t="inlineStr">
         <is>
-          <t>Base: 0.00s | FT Guided: 60.03s</t>
+          <t>Base: 0.00s | FT Guided: 108.15s</t>
         </is>
       </c>
       <c r="K78" s="4" t="inlineStr">
@@ -8398,17 +8521,39 @@
       </c>
       <c r="H79" s="4" t="inlineStr">
         <is>
-          <t>Error: HTTPConnectionPool(host='localhost', port=11434): Read timed out. (read timeout=60)</t>
-        </is>
-      </c>
-      <c r="I79" s="6" t="inlineStr">
-        <is>
-          <t>Low</t>
+          <t>Okay, let’s analyze this surveillance scene based on the provided activity class: “A person wearing gloves and a hat is reaching down into a trash can.”
+**What is happening?**
+The video shows an individual, obscured by a hat and gloves, actively reaching into a large trash can. They appear to be rummaging through the contents of the bin. 
+**Which activities are visible?**
+* **Reaching:** The primary activity is the deliberate act of reaching down into the trash can.
+* **Searching/Rummaging:**  The way they’re moving suggests they're looking for something within the waste.
+* **Presence in a Domestic Setting:** We see a decorated interior, indicating this likely takes place in a home or apartment.
+**Is there any suspicious behaviour?**
+Yes, there is definitely suspicious behavior. Reaching into a trash can, especially with gloves and a hat to conceal identity, raises immediate concerns. It’s not a typical action for someone simply discarding waste. 
+**Are there any threat indicators?**
+Several elements suggest potential threats:
+* **Concealed Identity:** The use of a hat and gloves is highly unusual and intended to obscure the individual's face.
+* **Trash Can Location:** Trash cans are often overlooked or less monitored areas within a property, making them attractive targets for illicit activity. 
+* **Unusual Action:**  The specific action – reaching into a trash can – is not routine and warrants scrutiny.
+**Estimate the threat level as Low, Medium, or High.**
+I would rate this threat level as **Medium**. 
+**Explain your reasoning:**
+While the individual’s actions are clearly suspicious, there isn't immediate evidence of violence or an obvious criminal intent. However, the combination of concealment and the unusual activity creates a significant risk. It could be:
+*   **Theft in Progress:** They might be searching for stolen items discarded by someone else.
+*   **Pre-Planning:** This could be reconnaissance – observing the property before attempting a more serious intrusion. 
+*   **Other Malicious Intent:** The activity could be part of a larger, unknown plan.
+**Recommendations:**
+This footage should be immediately reviewed by security personnel or law enforcement. Further investigation is crucial to determine the individual's identity, their purpose in accessing the trash can, and whether they pose an ongoing threat.  It would be beneficial to check for any other surveillance cameras that might have captured more of the event or the person’s movements before and after.</t>
+        </is>
+      </c>
+      <c r="I79" s="5" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
       <c r="J79" s="3" t="inlineStr">
         <is>
-          <t>Base: 0.00s | FT Guided: 60.02s</t>
+          <t>Base: 0.00s | FT Guided: 92.88s</t>
         </is>
       </c>
       <c r="K79" s="4" t="inlineStr">
@@ -8435,7 +8580,33 @@
       </c>
       <c r="D80" s="4" t="inlineStr">
         <is>
-          <t>Error: HTTPConnectionPool(host='localhost', port=11434): Read timed out. (read timeout=60)</t>
+          <t>Okay, let's analyze this surveillance video sequence.
+**What is happening?**
+The video shows a significant disruption to an entrance of what appears to be a shop or business. A large map has been forcefully pushed through the glass door and into the interior space. There’s a black car parked outside, and it seems like the event just occurred or is in its immediate aftermath. 
+**Which activities are visible?**
+* **Forceful Entry:** The primary activity is the forceful entry of a large map through the shop's front door.
+* **Vehicle Presence:** A dark-colored (likely black) car is parked outside, potentially related to the event or simply present at the time. 
+* **Interior Observation:** We can see some interior elements – shelving units with products, posters on the wall, and a handrail.
+**Is there any suspicious behaviour?**
+Yes, there’s definitely suspicious behavior. The way the map is being pushed through the door suggests an intentional act of damage or disruption rather than accidental movement. 
+**Are there any threat indicators?**
+* **Damage to Property:**  The broken glass and damaged door represent a clear breach of security and potential property damage.
+* **Potential for Further Action:** The event could be part of a larger operation, such as robbery or vandalism. The presence of the car adds an element of concern. 
+* **Disruption:** The disruption to business operations is itself a threat – potentially causing loss of revenue, inconvenience to customers, and damage to reputation.
+**Estimate the Threat Level as Low, Medium, or High.**
+I would estimate the threat level as **Medium**. 
+**Explanation of Reasoning:**
+Here’s why I've assigned a medium threat level:
+* **Not Immediately Violent:** The video doesn't show any immediate violence or threats directed at people. However, the forceful entry is concerning.
+* **Potential for Escalation:**  The act itself suggests an intent to cause damage and disruption. This could escalate into more serious criminal activity (theft, assault) if not addressed quickly. 
+* **Uncertain Motive:** We don't know *why* this happened. It could be random vandalism, a targeted attack, or part of something larger.  This uncertainty increases the risk.
+**Recommendations:**
+1. **Secure the Scene:** Immediately secure the area to prevent further damage and potential access for others.
+2. **Assess Damage:** Evaluate the extent of the damage to the door and glass. 
+3. **Review Surveillance Footage:** Thoroughly review all available surveillance footage to identify the individual(s) involved, their vehicle (if possible), and any other relevant details.
+4. **Contact Law Enforcement:**  Report the incident to the police immediately and provide them with the video evidence.
+**Disclaimer:** *This analysis is based solely on a still image provided. A full review of the video sequence would likely reveal more information and potentially alter my assessment.* 
+Would you like me to elaborate on any specific aspect of this analysis, or perhaps consider what additional information might be helpful in assessing the situation further?</t>
         </is>
       </c>
       <c r="E80" s="4" t="inlineStr">
@@ -8459,17 +8630,44 @@
       </c>
       <c r="H80" s="4" t="inlineStr">
         <is>
-          <t>Error: HTTPConnectionPool(host='localhost', port=11434): Read timed out. (read timeout=60)</t>
-        </is>
-      </c>
-      <c r="I80" s="6" t="inlineStr">
-        <is>
-          <t>Low</t>
+          <t>Okay, let’s analyze this surveillance footage based on the provided activity class and visual information.
+**What is happening?**
+The primary event is a vehicle crash through the glass entrance of a store. The force of the impact has shattered the glass door and caused damage to the surrounding area. It appears to be an active incident, as the car is still present in the scene. 
+**Which activities are visible?**
+* **Vehicle Impact:** The most prominent activity is the vehicle colliding with the storefront.
+* **Structural Damage:**  The destruction of the glass door and potential damage to the interior structure is evident.
+* **Presence of a Vehicle:** A dark-colored car (likely an Audi, based on the wheels) is parked outside the store, seemingly involved in the incident. 
+* **Store Interior Elements:** We can see elements within the store like shelving units, posters and other displays.
+**Is there any suspicious behaviour?**
+It's difficult to definitively determine suspicious behavior from a single frame of this video. However, the sudden and forceful impact suggests an unplanned event.  Without more context (e.g., audio), it’s impossible to say if this was intentional or accidental. 
+**Are there any threat indicators?**
+* **Damage:** The significant damage indicates a potential for injury to people inside or outside the store, as well as property damage.
+* **Vehicle Presence:**  The vehicle itself is a potential hazard and could be used in further actions. 
+* **Uncontrolled Event:** The sudden nature of the crash suggests an uncontrolled situation.
+**Estimate the threat level as Low, Medium, or High.**
+I would rate the threat level as **Medium**. 
+**Reasoning:**
+Here’s why I've assessed it as medium:
+*   **Potential for Injury:** The crash clearly presents a risk of injury to anyone nearby.
+*   **Property Damage:** Significant damage to the store is a concern, leading to potential business disruption and costs.
+*   **Uncertainty:** We don’t know the circumstances surrounding the crash (e.g., was it an accident, vandalism, or something else?). This uncertainty elevates the threat level slightly. 
+However, without further information (like audio from the scene, witness statements, or a clearer view of the vehicle's actions), it doesn’t immediately appear to be a high-risk situation like a violent assault. 
+**Further Investigation Needed:**
+It is crucial to gather more information:
+*   Review additional footage to understand the sequence of events leading up to the crash.
+*   Check for any injuries or casualties.
+*   Investigate the circumstances surrounding the incident (e.g., determine if it was an accident, vandalism, or a criminal act). 
+Do you want me to focus on describing specific elements within the image in more detail, such as the type of vehicle, the layout of the store, or any other details that might be relevant?</t>
+        </is>
+      </c>
+      <c r="I80" s="5" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
       <c r="J80" s="3" t="inlineStr">
         <is>
-          <t>Base: 60.04s | FT Guided: 60.04s</t>
+          <t>Base: 106.52s | FT Guided: 102.86s</t>
         </is>
       </c>
       <c r="K80" s="4" t="inlineStr">
@@ -8520,17 +8718,38 @@
       </c>
       <c r="H81" s="4" t="inlineStr">
         <is>
-          <t>Error: HTTPConnectionPool(host='localhost', port=11434): Read timed out. (read timeout=60)</t>
-        </is>
-      </c>
-      <c r="I81" s="6" t="inlineStr">
-        <is>
-          <t>Low</t>
+          <t>Okay, let’s analyze this surveillance scene based on the provided activity class and visual information.
+**What is happening?**
+The video shows a group of people gathered around a counter in what appears to be a restaurant or food service area. They are seated at tables and appear to be interacting with staff. It looks like they are either ordering, eating, or engaging in some other activity related to the establishment’s services. 
+**Which activities are visible?**
+*   **People Gathering:** Several individuals are present, clustered around a counter.
+*   **Interaction with Staff:**  There's evidence of interaction between customers and what appears to be restaurant staff (likely taking orders or serving food).
+*   **Seating:** People are seated at tables, suggesting they’re consuming food or drinks. 
+**Is there any suspicious behaviour?**
+Based on the single frame provided, it is difficult to determine if there is any suspicious behavior. However, we can note:
+*   The group appears relatively large – this could be a normal gathering, but warrants further observation in subsequent frames.
+*   There's no obvious indication of conflict or unusual movement within the group itself. 
+**Are there any threat indicators?**
+There are currently no immediately apparent threat indicators in this single frame. There is nothing overtly threatening about the scene. However, it’s important to note that a single frame provides limited context. 
+**Estimate the threat level as Low, Medium, or High.**
+Threat Level: **Low**
+**Reasoning:**
+The scene depicts a typical restaurant environment. The people are engaged in normal activities. There is no obvious violence, weapons, or other indicators of imminent danger.  However, it's crucial to understand that this assessment is based on *one* frame. A longer video sequence would be needed to fully assess the situation and identify any potential risks. 
+**Recommendations for Further Analysis:**
+*   **Review Subsequent Frames:** The most important step is to analyze additional frames of the video to observe movement patterns, interactions between individuals, and any changes in behavior over time.
+*   **Check for Unusual Activity:** Look for anything out of place – sudden movements, arguments, concealment of objects, or unusual groupings of people. 
+*   **Contextual Information:**  Gather information about the establishment (e.g., type of restaurant, typical clientele) to help interpret the scene.
+Would you like me to elaborate on any specific aspect of this analysis, such as potential areas for further investigation based on what we might expect to see in subsequent frames?</t>
+        </is>
+      </c>
+      <c r="I81" s="5" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
       <c r="J81" s="3" t="inlineStr">
         <is>
-          <t>Base: 0.00s | FT Guided: 60.02s</t>
+          <t>Base: 0.00s | FT Guided: 95.97s</t>
         </is>
       </c>
       <c r="K81" s="4" t="inlineStr">
@@ -8581,17 +8800,35 @@
       </c>
       <c r="H82" s="4" t="inlineStr">
         <is>
-          <t>Error: HTTPConnectionPool(host='localhost', port=11434): Read timed out. (read timeout=60)</t>
-        </is>
-      </c>
-      <c r="I82" s="6" t="inlineStr">
-        <is>
-          <t>Low</t>
+          <t>Okay, let’s analyze this surveillance scene based on the provided activity class and visual information.
+**What is happening?**
+The video shows a single individual seated at a desk, actively using a computer with a monitor. They appear to be engaged in some form of work or task related to the computer. Behind them, a display case containing candy and snacks is prominently visible. 
+**Which activities are visible?**
+* **Computer Use:** The primary activity is the individual operating a computer.
+* **Work/Task Performance:**  The person at the desk suggests they are engaged in some kind of work or task – we can’t determine exactly what it is from this frame alone, but it's an active engagement with the computer.
+* **Retail Observation:** The presence of the candy and snack display case indicates a retail environment (likely a convenience store or similar).
+**Is there any suspicious behaviour?**
+Based solely on this single frame, there isn’t immediately obvious *suspicious* behavior. However, the situation warrants careful observation. 
+**Are there any threat indicators?**
+The most notable potential threat indicator is the display case filled with candy and snacks. This could be a target for theft or robbery. The individual's position relative to this display case is also relevant – they are close enough to potentially access it easily.  The fact that the monitor is on, while not inherently threatening, suggests someone is actively engaged in something, which could be related to the potential threat.
+**Estimate the threat level as Low, Medium, or High.**
+I would rate the threat level as **Medium**. 
+**Reasoning:**
+* **Low Threat Factors:** The individual appears to be simply working at a computer. There's no obvious aggressive behavior or indication of intent.
+* **Medium Threat Factors:** The presence of a valuable retail display (candy/snacks) creates a potential vulnerability.  The person’s proximity to this display raises concerns about opportunistic theft. 
+* **Lack of Immediate Danger:** We don’t see any weapons, violence, or other immediate threats in this single frame.
+**Important Note:** This assessment is based on *one* frame of video. A more comprehensive analysis would require reviewing the entire sequence for patterns, movement, interactions with others, and changes in behavior over time.  It's crucial to consider context (time of day, location, known security protocols) when evaluating this scene. 
+Do you want me to elaborate on any specific aspect of this analysis, such as potential vulnerabilities or what further information would be helpful for a more thorough assessment?</t>
+        </is>
+      </c>
+      <c r="I82" s="5" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
       <c r="J82" s="3" t="inlineStr">
         <is>
-          <t>Base: 0.00s | FT Guided: 60.01s</t>
+          <t>Base: 0.00s | FT Guided: 95.09s</t>
         </is>
       </c>
       <c r="K82" s="4" t="inlineStr">
@@ -8642,17 +8879,43 @@
       </c>
       <c r="H83" s="4" t="inlineStr">
         <is>
-          <t>Error: HTTPConnectionPool(host='localhost', port=11434): Read timed out. (read timeout=60)</t>
-        </is>
-      </c>
-      <c r="I83" s="6" t="inlineStr">
-        <is>
-          <t>Low</t>
+          <t>Okay, let’s analyze this surveillance scene based on the provided activity class: “A man is attempting to rob a shop by using a crowbar to force open the entrance.”
+**What is happening?**
+The video depicts an individual actively trying to break into a retail establishment – likely a small shop or convenience store. The primary action is the forceful entry attempt using a crowbar against the door. 
+**Which activities are visible?**
+*   **Robbery Attempt:** The core activity is the deliberate and aggressive effort to gain unauthorized access with the intent of theft (likely).
+*   **Crowbar Use:**  The individual is actively wielding and applying force with a crowbar to damage the door’s locking mechanism or frame.
+*   **Presence of Vehicles:** Several vehicles are visible in the background, suggesting this activity is taking place on a street or near a road. One appears to be a police vehicle. 
+*   **Security Camera Presence:** The presence of a security camera itself indicates an attempt at concealment and potentially a heightened awareness of surveillance.
+**Is there any suspicious behaviour?**
+Yes, absolutely. All the elements combine to create highly suspicious behavior:
+*   **Targeted Action:**  The focused effort on the shop entrance is not random; it’s a deliberate targeting of property for potential theft.
+*   **Use of Force:** Employing a crowbar to force entry demonstrates an intent to overcome security measures and poses immediate physical danger. 
+*   **Timing (Implied):** The fact that this is captured on surveillance suggests the individual may have been aware of camera coverage, adding another layer of suspiciousness.
+**Are there any threat indicators?**
+Yes, several:
+*   **Potential for Physical Harm:** The use of a crowbar presents a significant risk of injury to anyone inside or nearby.
+*   **Theft Risk:**  The primary goal is likely theft, which can have serious financial consequences for the business owner and potential harm to customers. 
+*   **Escalation Potential:** Robbery attempts often escalate into violence if resisted.
+**Estimate the threat level as Low, Medium, or High.**
+I would rate this threat level as **High**.
+**Reasoning:**
+Here’s why I assess it as high:
+1.  **Direct Threat of Force:** The use of a crowbar immediately elevates the risk to a dangerous level. It's not just a potential for theft; it's an active attempt to cause damage and potentially harm someone.
+2.  **Intentional Criminal Act:** Robbery is inherently a serious crime with significant consequences. 
+3.  **Unpredictability:** Robbery attempts can quickly escalate, making them unpredictable and dangerous. The presence of a police vehicle in the background suggests an immediate response is likely, but that doesn't negate the ongoing threat.
+It’s crucial to note that this assessment is based solely on the visual information provided. Further investigation would be needed to confirm details and assess the full extent of the situation. 
+Do you want me to focus on a specific aspect of this analysis (e.g., the individual's appearance, the surrounding environment, or potential follow-up actions)?</t>
+        </is>
+      </c>
+      <c r="I83" s="5" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
       <c r="J83" s="3" t="inlineStr">
         <is>
-          <t>Base: 0.00s | FT Guided: 60.01s</t>
+          <t>Base: 0.00s | FT Guided: 109.28s</t>
         </is>
       </c>
       <c r="K83" s="4" t="inlineStr">
@@ -8703,7 +8966,35 @@
       </c>
       <c r="H84" s="4" t="inlineStr">
         <is>
-          <t>Error: HTTPConnectionPool(host='localhost', port=11434): Read timed out. (read timeout=60)</t>
+          <t>Okay, let’s analyze this surveillance scene based on the provided activity class and visual evidence.
+**What is happening?**
+The video shows a man rapidly exiting a store in a hurry. He appears to be engaged in a phone conversation while doing so. A second individual stands behind him, seemingly observing or following. 
+**Which activities are visible?**
+* **Running/Rapid Movement:** The primary activity is the man’s quick departure from the store.
+* **Phone Conversation:**  He's actively speaking on his mobile phone.
+* **Following/Observation:** The second individual is standing behind him, suggesting observation or potential following. 
+* **Store Exit:** The scene takes place at a retail store entrance.
+**Is there any suspicious behaviour?**
+Yes, there is potentially suspicious behavior. The hurried exit, coupled with the phone conversation and the presence of another person observing, raises concerns. It’s not immediately obvious if this is normal or indicative of something illicit. 
+**Are there any threat indicators?**
+While we can't definitively determine a threat level from just this single frame, several elements suggest potential concern:
+* **Rapid Departure:** Often, hurried exits are associated with attempts to avoid detection or conceal an action.
+* **Phone Conversation:** The content of the conversation is unknown, but it could be related to illegal activities. 
+* **Presence of a Second Individual:**  This adds an element of uncertainty and potential risk.
+**Estimate the threat level as Low, Medium, or High.**
+I would estimate the threat level as **Medium**. 
+**Explain your reasoning:**
+My assessment is based on the combination of factors:
+*   **Uncertain Context:** We don't know *why* he’s running out of the store. It could be a legitimate reason (e.g., an emergency), but the circumstances are suspicious.
+*   **Potential for Concealment:** The hurried exit suggests he might be trying to avoid being seen or questioned. 
+*   **Presence of Observer:**  The second individual adds another layer of complexity and potential risk.
+It's not a high threat level because we lack concrete evidence of criminal activity (like weapons, violence, etc.). However, the combination of elements warrants further investigation and monitoring to determine if this is simply unusual behavior or something more concerning. 
+**Further Investigation Needed:**
+To get a clearer picture, it would be crucial to:
+*   Analyze additional frames in the video sequence for context.
+*   Identify the second individual – who are they? What is their relationship to the man running out of the store?
+*   Determine the content of the phone conversation (if possible). 
+Would you like me to focus on describing any specific elements within the image, such as details about the individuals or the store environment?</t>
         </is>
       </c>
       <c r="I84" s="6" t="inlineStr">
@@ -8713,7 +9004,7 @@
       </c>
       <c r="J84" s="3" t="inlineStr">
         <is>
-          <t>Base: 0.00s | FT Guided: 60.03s</t>
+          <t>Base: 0.00s | FT Guided: 101.61s</t>
         </is>
       </c>
       <c r="K84" s="4" t="inlineStr">
@@ -8740,7 +9031,28 @@
       </c>
       <c r="D85" s="4" t="inlineStr">
         <is>
-          <t>Error: HTTPConnectionPool(host='localhost', port=11434): Read timed out. (read timeout=60)</t>
+          <t>Okay, let's analyze this surveillance video sequence based on the image provided.
+**What is happening?**
+The scene depicts a confrontation between a man in a white cap and a driver of a white van. The man appears to be attempting to physically impede the vehicle’s movement by grabbing onto it.  It looks like an attempt to stop or block the van. 
+**Which activities are visible?**
+*   **Man's Action:** A man is actively trying to grab and hold onto the side of a white van, pulling against it.
+*   **Driver’s Reaction:** The driver of the van appears startled and is reacting defensively.
+*   **Vehicle Movement:** The van is attempting to move forward despite the man's interference. 
+**Is there any suspicious behaviour?**
+Yes, there is definitely suspicious behavior. The man’s deliberate action of grabbing onto a moving vehicle raises immediate concerns. It isn't a normal or expected interaction.
+**Are there any threat indicators?**
+*   **Physical Contact:** The direct physical contact between the man and the van represents a potential for harm.
+*   **Intentional Action:** The man’s deliberate attempt to impede the vehicle suggests an intention to disrupt its movement, which could escalate into more serious actions. 
+*   **Unpredictability:**  The situation is inherently unpredictable due to the sudden intervention of the man.
+**Estimate the threat level as Low, Medium, or High.**
+I would estimate the threat level as **Medium**.
+**Explanation of Reasoning:**
+Here’s why I've assigned a medium threat level:
+*   **Not Immediately Violent:**  As of this image, there is no indication of violence (no punches thrown, etc.). However, the action itself – deliberately grabbing onto a moving vehicle – creates a significant potential for escalation.
+*   **Unclear Motivation:** We don't know *why* the man is doing this. It could be a road rage incident, an attempt to prevent something within the van, or something else entirely. This uncertainty increases the risk. 
+*   **Potential for Escalation:** The situation has the potential to quickly become more dangerous if either party reacts aggressively.  The driver might feel threatened and respond defensively.
+**Important Note:** *This analysis is based solely on a single image from a surveillance video sequence.* A full review of the video would be necessary to fully understand the context, motivations, and overall threat level. It's crucial to consider factors like body language, surrounding environment, and any other visible details that might provide additional clues. 
+Would you like me to elaborate on any specific aspect of this analysis or discuss what further information would be helpful in assessing the situation more thoroughly?</t>
         </is>
       </c>
       <c r="E85" s="4" t="inlineStr">
@@ -8762,17 +9074,43 @@
       </c>
       <c r="H85" s="4" t="inlineStr">
         <is>
-          <t>Error: HTTPConnectionPool(host='localhost', port=11434): Read timed out. (read timeout=60)</t>
-        </is>
-      </c>
-      <c r="I85" s="6" t="inlineStr">
-        <is>
-          <t>Low</t>
+          <t>Okay, let’s analyze this surveillance scene based on the provided activity class and visual evidence.
+**What is happening?**
+The video depicts a situation where one man is actively attempting to push a white van, while another man stands nearby watching. It appears to be an attempt to move or potentially immobilize the vehicle. 
+**Which activities are visible?**
+* **Pushing:** The primary activity is the forceful pushing of the van by one individual.
+* **Observation/Watching:**  The second individual is standing and observing the action, seemingly taking note of what's happening.
+* **Vehicle Movement (attempted):** The van itself is being subjected to a push, indicating an attempt to move it. 
+**Is there any suspicious behaviour?**
+Yes, there is potentially suspicious behavior. The deliberate act of pushing a vehicle, especially with another person observing, raises concerns. It’s not immediately clear what the motive is, but this action isn't typical and warrants further scrutiny. 
+**Are there any threat indicators?**
+Several elements suggest potential threats:
+* **Forceful Action:** Pushing a vehicle can be interpreted as an aggressive act or an attempt to cause damage or disruption.
+* **Presence of a Witness:** The second individual observing adds another layer of complexity and could indicate involvement, coordination, or simply observation for later use. 
+* **Unclear Motive:**  The lack of context makes it difficult to determine the intent behind this action.
+**Estimate the threat level as Low, Medium, or High.**
+I would rate the threat level as **Medium**. 
+**Reasoning:**
+Here’s why I've assigned a medium threat level:
+* **Not Immediately Violent:** The pushing itself isn't inherently violent. It could be a misguided attempt to move the van for some reason (perhaps a misunderstanding or a prank gone wrong).
+* **Potential for Escalation:** However, the deliberate nature of the action and the presence of an observer suggest that this could escalate into something more serious. The intent is unclear, and there's a possibility it’s part of a larger plan. 
+* **Need for Investigation:**  The situation requires immediate investigation to determine the motive behind the pushing, the role of the second individual, and whether any further actions are planned.
+**Recommendations:**
+Based on this analysis, I recommend:
+1.  **Immediate Review of Surveillance Footage:** Thoroughly examine the surrounding footage to identify the individuals involved, their movements before, during, and after the event, and any potential vehicles or persons of interest nearby.
+2. **Contact Law Enforcement:** Report the incident to local law enforcement for investigation. 
+3. **Determine Motive:**  Investigate the reason behind the pushing – was it a misunderstanding, vandalism, or part of a criminal scheme?
+Do you want me to elaborate on any specific aspect of this analysis, such as potential motives or recommended investigative steps?</t>
+        </is>
+      </c>
+      <c r="I85" s="5" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
       <c r="J85" s="3" t="inlineStr">
         <is>
-          <t>Base: 60.02s | FT Guided: 60.02s</t>
+          <t>Base: 96.92s | FT Guided: 104.43s</t>
         </is>
       </c>
       <c r="K85" s="4" t="inlineStr">
@@ -8823,17 +9161,41 @@
       </c>
       <c r="H86" s="4" t="inlineStr">
         <is>
-          <t>Error: HTTPConnectionPool(host='localhost', port=11434): Read timed out. (read timeout=60)</t>
-        </is>
-      </c>
-      <c r="I86" s="6" t="inlineStr">
-        <is>
-          <t>Low</t>
+          <t>Okay, let’s analyze this surveillance scene based on the provided activity class and visual evidence.
+**What is happening?**
+The video depicts a violent assault in progress. A man is being attacked by multiple individuals, resulting in him falling to the ground. The scene appears chaotic with several people present, some of whom are actively involved in the attack or reacting to it. 
+**Which activities are visible?**
+*   **Attack:** The primary activity is a physical assault – a man is being forcefully struck and pushed to the ground.
+*   **Reaction/Response:** Several individuals are observing the event, some appear to be running away, while others are standing around seemingly watching or reacting. 
+*   **Movement:** There’s movement from multiple people in the scene - running, approaching, and surrounding the victim.
+**Is there any suspicious behaviour?**
+Yes, several elements suggest suspicious behavior:
+*   **Group Dynamics:** The presence of a group of individuals engaged in this activity is inherently suspicious. It suggests an organized or coordinated attack.
+*   **Lack of Immediate Intervention:** While some people are moving away, the lack of immediate intervention by others raises questions about their involvement or awareness. 
+*   **Positioning:** Some individuals are positioned to observe the event closely, which could indicate they are involved or have a vested interest.
+**Are there any threat indicators?**
+Absolutely. The key threat indicators include:
+*   **Physical Violence:** The core indicator is the violent attack itself – physical harm is being inflicted.
+*   **Multiple Perpetrators:** The involvement of multiple individuals significantly increases the potential for escalation and further violence. 
+*   **Unclear Intentions:** Without context, it's difficult to determine the motive behind the attack, but the aggressive nature suggests a serious threat.
+**Estimate the Threat Level as Low, Medium, or High.**
+I would estimate the threat level as **Medium**.
+**Reasoning:**
+Here’s why I assess the threat level as medium:
+*   **Severity of Action:** The act of violent assault is inherently dangerous and carries a significant risk of serious injury.
+*   **Number of Involved Parties:** While not a large group, the involvement of multiple individuals increases the potential for escalation and further harm. 
+*   **Uncertainty:** Without knowing the motive or relationship between the parties involved, it's difficult to assess the long-term threat. It could be a spontaneous act of aggression, but the coordinated nature suggests something more deliberate.
+**Important Disclaimer:** *I want to reiterate that this analysis is based solely on the visual information provided in the image and the activity class description. I do not endorse or condone violence in any way.*  A full investigation would require much more context, including witness statements, background information about the individuals involved, and a determination of the motive for the attack.</t>
+        </is>
+      </c>
+      <c r="I86" s="5" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
       <c r="J86" s="3" t="inlineStr">
         <is>
-          <t>Base: 0.00s | FT Guided: 60.03s</t>
+          <t>Base: 0.00s | FT Guided: 101.19s</t>
         </is>
       </c>
       <c r="K86" s="4" t="inlineStr">
@@ -8884,7 +9246,35 @@
       </c>
       <c r="H87" s="4" t="inlineStr">
         <is>
-          <t>Error: HTTPConnectionPool(host='localhost', port=11434): Read timed out. (read timeout=60)</t>
+          <t>Okay, let’s analyze this surveillance scene based on the provided activity class and visual evidence.
+**What is happening?**
+The image depicts a highly chaotic and potentially volatile situation unfolding on a cobblestone street at night. There's a large crowd present, and police officers are actively engaged in attempting to manage or control that crowd. The overall impression is one of disruption and an event having just occurred (as suggested by the activity class). 
+**Which activities are visible?**
+* **Crowd Movement:** People are moving erratically throughout the scene – some running, others standing still, and a general sense of disarray within the crowd.
+* **Police Intervention:** Several police officers are visible, seemingly attempting to direct traffic, separate individuals, or establish a perimeter. They appear to be actively engaging with the crowd. 
+* **Barrier Presence:** A temporary barrier (orange cone) is present, likely deployed by law enforcement to control movement and potentially protect an area.
+* **Street Scene:** The cobblestone street itself provides context – it’s a public space where this event is taking place.
+**Is there any suspicious behaviour?**
+It's difficult to definitively identify specific "suspicious behaviors" from just this single frame, but several elements raise concerns:
+* **Uncontrolled Crowd:** The sheer size and lack of order within the crowd itself could be considered a potential indicator of unrest or an uncontrolled reaction to something.
+* **Individual Reactions:** Some individuals appear agitated or are looking around intensely – these reactions could be linked to the incident or simply a response to the chaos. 
+**Are there any threat indicators?**
+While not immediately obvious from this single frame, several factors suggest potential threats:
+* **Police Presence:** The significant number of police officers indicates that something has escalated beyond a normal situation and requires a controlled response.
+* **Crowd Dynamics:**  The movement of the crowd suggests a possible loss of control, which can quickly lead to dangerous situations (e.g., stampedes). 
+* **Unidentified Incident:** The activity class mentions “what appears to be an incident,” implying that something has triggered this reaction. Without knowing what that was, it’s impossible to fully assess the threat level.
+**Estimate the Threat Level as Low, Medium, or High.**
+I would estimate the threat level as **Medium**. 
+**Reasoning:**
+* **Not Imminent Violence (Low):** There's no visible evidence of direct violence (e.g., weapons being brandished, someone actively attacking).
+* **Potential for Escalation (Medium):** The chaotic crowd and police intervention suggest a situation that *could* escalate into more serious incidents – riots, injuries, or further unrest.  The “incident” mentioned in the activity class adds to this concern. 
+* **Uncertainty (Important Consideration):** The unknown nature of the initial incident is a significant factor driving the threat level up. Until we know what triggered this response, there’s an inherent risk that things could worsen rapidly.
+**Further Investigation Needed:**
+To refine this assessment, it would be crucial to:
+*   Identify the cause of the incident.
+*   Analyze additional frames from the video sequence to understand the progression of events.
+*   Gather information about any reported injuries or damage. 
+Do you want me to elaborate on a specific aspect of this analysis (e.g., the role of the police, potential causes of the crowd reaction)?</t>
         </is>
       </c>
       <c r="I87" s="6" t="inlineStr">
@@ -8894,7 +9284,7 @@
       </c>
       <c r="J87" s="3" t="inlineStr">
         <is>
-          <t>Base: 0.00s | FT Guided: 60.01s</t>
+          <t>Base: 0.00s | FT Guided: 114.23s</t>
         </is>
       </c>
       <c r="K87" s="4" t="inlineStr">
@@ -8945,17 +9335,35 @@
       </c>
       <c r="H88" s="4" t="inlineStr">
         <is>
-          <t>Error: HTTPConnectionPool(host='localhost', port=11434): Read timed out. (read timeout=60)</t>
-        </is>
-      </c>
-      <c r="I88" s="6" t="inlineStr">
-        <is>
-          <t>Low</t>
+          <t>Okay, let’s analyze this surveillance scene based on the provided activity class and visual evidence.
+**What is happening?**
+The image depicts a violent assault occurring within an internet cafe. A man is aggressively attacking individuals who are seated at computers. The scene quickly escalates into widespread chaos as people react to the attack. 
+**Which activities are visible?**
+*   **Attack:** The primary activity is a physical assault where one individual (the attacker) is violently striking multiple others.
+*   **Reaction/Flight:** Individuals seated at the computers are reacting with surprise, fear, and attempting to flee or defend themselves. Some appear to be moving away from the immediate area of the attack.
+*   **Observation:** Several individuals are observing the event unfold, some appearing shocked or concerned. 
+*   **Computer Use (Pre-Attack):** Before the assault, people are visibly using computers at their workstations.
+**Is there any suspicious behaviour?**
+While it's difficult to determine specific pre-attack behavior from a single frame, the overall scene suggests a sudden and unexpected escalation of violence. The attacker’s actions are clearly not normal or expected behavior in an internet cafe setting. 
+**Are there any threat indicators?**
+*   **Aggressive Posture:** The attacker's body language is aggressive – he is moving towards the victims with intent to harm.
+*   **Physical Contact:** The direct physical contact between the attacker and the victims indicates a serious threat of injury.
+*   **Disruption of Order:** The attack immediately disrupts the normal operation of the internet cafe, creating an unsafe environment for everyone present. 
+**Estimate the Threat Level as Low, Medium, or High.**
+**High**. 
+**Reasoning:**
+The image clearly shows a violent assault in progress with multiple victims involved. The attacker’s aggressive actions and the resulting chaos represent a significant threat to the safety of those present.  The potential for further violence is high given the initial escalation. While we don't have context about the attacker's motives or whether this was a targeted attack, the immediate danger posed by the assault warrants a high threat level assessment. 
+**Important Note:** This analysis is based solely on the provided image and the activity class description. A more comprehensive understanding would require reviewing additional frames of the video sequence, analyzing audio data (if available), and gathering contextual information about the event.</t>
+        </is>
+      </c>
+      <c r="I88" s="5" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
       <c r="J88" s="3" t="inlineStr">
         <is>
-          <t>Base: 0.00s | FT Guided: 60.03s</t>
+          <t>Base: 0.00s | FT Guided: 91.25s</t>
         </is>
       </c>
       <c r="K88" s="4" t="inlineStr">
@@ -9006,17 +9414,45 @@
       </c>
       <c r="H89" s="4" t="inlineStr">
         <is>
-          <t>Error: HTTPConnectionPool(host='localhost', port=11434): Read timed out. (read timeout=60)</t>
-        </is>
-      </c>
-      <c r="I89" s="6" t="inlineStr">
-        <is>
-          <t>Low</t>
+          <t>Okay, let’s analyze this surveillance scene based on the provided activity class and visual evidence.
+**What is happening?**
+The video shows a group of people surrounding a fallen motorcycle in what appears to be an automotive garage or repair shop. They are actively observing the damage to the bike and seem to be trying to determine how it fell over. It’s likely they're assessing the extent of the damage, potentially looking for clues about the cause (e.g., mechanical failure, accident), and possibly planning a repair.
+**Which activities are visible?**
+* **Observation:** The primary activity is the group observing the motorcycle and its damage.
+* **Assessment:** Individuals are examining the bike closely, likely checking for broken parts or signs of impact. 
+* **Discussion/Communication:**  The people are standing in a circle, suggesting they're talking to each other about what happened and how to proceed.
+* **Potential Investigation:** Someone (likely the person with the flashlight) is shining it on the motorcycle and surrounding area, indicating an attempt to find clues or evidence.
+**Is there any suspicious behaviour?**
+There are a few elements that warrant closer scrutiny:
+* **Group Dynamics:** The fact that several people are gathered together could be normal for assessing damage, but it also raises questions about whether they're coordinating something.
+* **Flashlight Use:**  The use of a flashlight to examine the motorcycle is slightly unusual and could indicate an attempt to conceal evidence or obscure details. 
+**Are there any threat indicators?**
+While not overtly threatening, the situation does present some potential concerns:
+* **Unexplained Incident:** A fallen motorcycle suggests an accident or malfunction. The circumstances surrounding this event are unknown.
+* **Potential for Concealment:**  The flashlight and group dynamics raise the possibility that something isn't being disclosed – perhaps a deliberate act caused the fall, or there’s something they’re trying to hide about the damage.
+**Estimate the threat level as Low, Medium, or High.**
+I would rate the threat level as **Medium**. 
+**Explain your reasoning:**
+My assessment of ‘Medium’ is based on the following:
+*   **Uncertainty:** The core issue – a fallen motorcycle – is inherently suspicious. We don't know *why* it fell, and that uncertainty creates potential for wrongdoing.
+*   **Group Behavior:** While not necessarily malicious, the group dynamic and flashlight use introduce an element of concern. It’s possible they are covering something up or involved in something illicit. 
+*   **Lack of Immediate Obvious Threat:** There's no visible violence or immediate danger. However, the situation is ripe for escalation if there's a hidden motive.
+**Further Investigation Needed:**
+This scene warrants further investigation. Specifically, I would want to:
+*   Review security footage from surrounding cameras to see who entered and exited the garage around the time of the incident.
+*   Investigate the history of the motorcycle (ownership, maintenance records).
+*   Interview all individuals involved to understand their accounts of what happened. 
+Do you want me to focus on a specific aspect of this scene for further analysis, such as the flashlight use or the group dynamics?</t>
+        </is>
+      </c>
+      <c r="I89" s="5" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
       <c r="J89" s="3" t="inlineStr">
         <is>
-          <t>Base: 0.00s | FT Guided: 60.02s</t>
+          <t>Base: 0.00s | FT Guided: 109.12s</t>
         </is>
       </c>
       <c r="K89" s="4" t="inlineStr">
@@ -9043,7 +9479,29 @@
       </c>
       <c r="D90" s="4" t="inlineStr">
         <is>
-          <t>Error: HTTPConnectionPool(host='localhost', port=11434): Read timed out. (read timeout=60)</t>
+          <t>Okay, let's analyze this surveillance video sequence.
+**What is happening?**
+The video shows a man standing in the middle of a Moscow Metro train carriage, performing a series of increasingly frantic and erratic movements – essentially a dance-like performance. He’s extending his arms, bending at the waist, and generally moving with an almost manic energy.  Several other passengers are present, appearing startled and uncomfortable by the situation.
+**Which activities are visible?**
+* **The Man's Performance:** The primary activity is the man’s unusual movement – a seemingly spontaneous dance within the confined space of the train.
+* **Passenger Reactions:** Passengers are seated, observing the man with expressions ranging from surprise to concern and discomfort. One passenger is filming with his phone. 
+* **Train Movement:**  The train is moving forward, as indicated by the blurred background.
+**Is there any suspicious behaviour?**
+Yes, absolutely. The man's behavior is highly unusual and disruptive in a public space like a subway car. His movements are not typical of someone simply seeking a seat or observing their surroundings. 
+**Are there any threat indicators?**
+While the immediate threat appears low, several factors raise concerns:
+* **Unpredictability:** The man's actions are completely unpredictable and could escalate.
+* **Disruption:** He is deliberately disrupting the normal operation of the train and causing distress to other passengers. 
+* **Potential for escalation:**  The intensity of his movements suggests a possible loss of control, which could lead to further erratic behavior or potentially harmful actions.
+**Estimate the threat level as Low, Medium, or High.**
+I would rate this threat level as **Medium**. 
+**Explanation of Reasoning:**
+Here’s why I've assessed it as medium:
+* **No Immediate Violence:** There is no visible physical violence or aggressive behavior displayed by the man. He isn't threatening anyone directly with words or actions.
+* **Potential for Escalation:** The key factor driving the "Medium" rating is the *potential* for escalation. His erratic movements suggest a possible mental health issue, and that could lead to unpredictable behaviour.  The fact that he’s performing in a public space adds another layer of risk – it's harder to control him if he becomes agitated.
+* **Disruption &amp; Distress:** The disruption he is causing to other passengers is a significant concern. 
+**Important Note:** This analysis is based solely on the visual information presented in the image. A full assessment would require additional context, such as knowing the man's background, mental state (if known), and any subsequent events that unfolded after this video was recorded.  It’s crucial to remember that a seemingly harmless situation can quickly become dangerous. 
+Would you like me to elaborate on any specific aspect of this analysis or consider alternative interpretations?</t>
         </is>
       </c>
       <c r="E90" s="4" t="inlineStr">
@@ -9065,17 +9523,44 @@
       </c>
       <c r="H90" s="4" t="inlineStr">
         <is>
-          <t>Error: HTTPConnectionPool(host='localhost', port=11434): Read timed out. (read timeout=60)</t>
-        </is>
-      </c>
-      <c r="I90" s="6" t="inlineStr">
-        <is>
-          <t>Low</t>
+          <t>Okay, let’s analyze this surveillance video sequence based on the provided activity class and visual evidence.
+**What is happening?**
+The core event is a highly unusual and dramatic action: a man abruptly leaps from a seated position on a Moscow subway train to stand upright in mid-air, seemingly for the purpose of taking a photograph. It’s a very theatrical and unexpected movement. 
+**Which activities are visible?**
+* **Leaping/Jumping:** The primary activity is the sudden, forceful leap.
+* **Sitting:** A man is initially seated on the train.
+* **Standing:**  The man transitions to standing after the jump.
+* **Photograph Taking (Implied):** The context suggests he was attempting to take a photograph of himself in this pose. 
+* **Passenger Observation:** Other passengers are present and observing the event, some with phones presumably recording it.
+**Is there any suspicious behaviour?**
+Yes, absolutely. The behavior is highly unusual and disruptive.  The deliberate, theatrical nature of the jump suggests an attempt to draw attention to himself and create a spectacle. This immediately raises suspicion. 
+**Are there any threat indicators?**
+While this specific action doesn't inherently represent a direct physical threat, several factors contribute to potential concern:
+* **Disruption:** The sudden movement disrupts the normal operation of public transport and causes distress to other passengers.
+* **Attention-Seeking Behavior:**  The act is clearly intended to be noticed, which can escalate into more problematic behavior if not addressed. 
+* **Potential for Escalation:** While unlikely in this isolated instance, such actions could potentially be part of a larger plan or indicate unstable mental state.
+**Estimate the threat level as Low, Medium, or High.**
+**Medium**. 
+**Explain your reasoning:**
+Here’s why I assess the threat level as medium:
+* **Low Physical Threat:** The immediate physical danger posed by this action is minimal – it's a jump and doesn't involve violence.
+* **Moderate Disruption &amp; Potential for Escalation:**  The behavior itself is disruptive, which can be unsettling to other passengers. More importantly, the attention-seeking nature of the act raises concerns about potential escalation if the individual were to engage in further erratic or disruptive behaviour. 
+* **Unpredictability:** The suddenness and lack of apparent reason behind the action make it difficult to assess the individual's intentions.
+**Recommendations (based on this analysis):**
+*  Train staff should be alerted to monitor the situation closely.
+*  Security personnel may want to discreetly observe the individual’s behavior after the event. 
+*  It would be prudent to investigate if the person is under the influence of something or has a history of erratic behaviour.
+Do you want me to focus on any specific aspect of this analysis, such as potential motivations or further recommendations?</t>
+        </is>
+      </c>
+      <c r="I90" s="5" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
       <c r="J90" s="3" t="inlineStr">
         <is>
-          <t>Base: 60.03s | FT Guided: 60.03s</t>
+          <t>Base: 97.92s | FT Guided: 100.20s</t>
         </is>
       </c>
       <c r="K90" s="4" t="inlineStr">
@@ -9126,17 +9611,43 @@
       </c>
       <c r="H91" s="4" t="inlineStr">
         <is>
-          <t>Error: HTTPConnectionPool(host='localhost', port=11434): Read timed out. (read timeout=60)</t>
-        </is>
-      </c>
-      <c r="I91" s="6" t="inlineStr">
-        <is>
-          <t>Low</t>
+          <t>Okay, let’s analyze this surveillance scene based on the provided activity class: “A man is aggressively attacking and wrestling with an employee inside a retail store, knocking over displays and equipment.”
+**What is happening?**
+The video depicts a violent confrontation between two individuals within a retail environment. A male suspect is actively engaging in a physical assault against a store employee. The action involves grappling, pushing, and forceful movements, resulting in the disruption of merchandise and store fixtures. 
+**Which activities are visible?**
+* **Physical Assault:** The primary activity is the aggressive attack by the suspect on the employee.
+* **Wrestling/Grappling:**  The suspect is actively wrestling with the employee, demonstrating a struggle for control.
+* **Property Damage:** Displays and equipment (shelves, possibly a stool) are being knocked over due to the force of the interaction. 
+* **Movement:** Both individuals are moving rapidly within the store space.
+**Is there any suspicious behaviour?**
+Yes, several elements suggest suspicious behavior prior to the assault:
+* **Initial Approach:** The video shows the suspect approaching the employee in a way that seems confrontational and potentially threatening.  His body language is tense.
+* **Aggressive Posture:** Before the physical contact, the suspect’s posture suggests intent or preparation for an aggressive action. 
+**Are there any threat indicators?**
+Absolutely. Several visual cues indicate a high level of threat:
+* **Physical Contact:** The direct physical assault itself represents a significant threat to the employee's safety and well-being.
+* **Forceful Movements:**  The suspect’s movements are forceful, indicating potential harm beyond simple pushing or shoving. 
+* **Disruption of Store Environment:** Knocking over displays creates a chaotic environment and increases the risk of further injury or escalation.
+**Estimate the threat level as Low, Medium, or High.**
+**High**. 
+**Explain your reasoning:**
+The combination of factors strongly indicates a high threat level:
+1. **Direct Assault:** The core activity is an aggressive attack, which inherently poses a serious risk of physical harm.
+2. **Forceful Interaction:**  The wrestling and pushing demonstrate the potential for significant injury.
+3. **Unpredictability:** The situation is highly unpredictable – the escalation could quickly lead to more severe consequences (e.g., serious injuries, further violence). 
+4. **Potential for Escalation:** A physical assault can easily escalate into other forms of criminal behavior or even a life-threatening situation.
+**Important Note:** This analysis is based solely on the provided image and the given activity class description.  A full investigation would require reviewing additional footage, gathering witness statements, and potentially consulting with law enforcement. 
+Would you like me to focus on any particular aspect of this analysis in more detail (e.g., specific body language cues, potential motives, or recommended response actions)?</t>
+        </is>
+      </c>
+      <c r="I91" s="5" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
       <c r="J91" s="3" t="inlineStr">
         <is>
-          <t>Base: 0.00s | FT Guided: 60.02s</t>
+          <t>Base: 0.00s | FT Guided: 100.64s</t>
         </is>
       </c>
       <c r="K91" s="4" t="inlineStr">
@@ -9187,17 +9698,43 @@
       </c>
       <c r="H92" s="4" t="inlineStr">
         <is>
-          <t>Error: HTTPConnectionPool(host='localhost', port=11434): Read timed out. (read timeout=60)</t>
-        </is>
-      </c>
-      <c r="I92" s="6" t="inlineStr">
-        <is>
-          <t>Low</t>
+          <t>Okay, let’s analyze this surveillance scene based on the provided activity class and visual evidence.
+**What is happening?**
+The video clearly shows a sudden and disruptive intrusion into an office environment. A man enters the room in a state of apparent panic or urgency, rapidly moving through workstations. This suggests a highly unexpected and potentially destabilizing event. 
+**Which activities are visible?**
+* **Intrusion:** The primary activity is the forceful entry of an individual into a secured workspace.
+* **Rapid Movement:** The man’s frantic movement across the desks indicates urgency, possibly fear or disorientation.
+* **Workstation Interaction:**  He interacts with multiple computer workstations, suggesting he's searching for something or attempting to access information. 
+* **Employee Reaction:** Other individuals in the office are reacting – some appear startled and look towards the intruder, while others seem to be observing the situation.
+**Is there any suspicious behaviour?**
+Yes, absolutely. The entire sequence is highly suspicious due to:
+* **Unannounced Entry:** Entering an office without authorization is a serious breach of security.
+* **Erratic Movement:**  The man’s panicked and rapid movement suggests he's not behaving normally or under control. This could indicate distress, disorientation, or intent to cause disruption. 
+* **Lack of Clear Purpose:** The video doesn’t show him interacting with anyone in a productive way; his actions are solely focused on moving through the workstations.
+**Are there any threat indicators?**
+While we can't definitively determine intent from this single frame, several elements raise potential threat concerns:
+* **Uncontrolled Movement:**  The man's frantic behavior could indicate he’s unstable or potentially dangerous.
+* **Disruption of Operations:** His actions are directly disrupting the normal operations of the office and creating a chaotic environment. 
+* **Potential for Harm:** The sudden intrusion creates an immediate risk of physical harm to employees or damage to property.
+**Estimate the threat level as Low, Medium, or High.**
+I would estimate the threat level as **Medium**. 
+**Reasoning:**
+Here’s why I've assigned a medium threat level:
+* **Unpredictability:** The situation is inherently unpredictable due to the man’s erratic behavior and unknown motives.
+* **Potential for Escalation:** While we don’t know his intentions, the intrusion itself creates an immediate risk of escalation – he could become confrontational, attempt to steal information, or cause further disruption. 
+* **Lack of Immediate Harm:** There's no visible evidence of violence or direct threat at this moment. However, the situation is volatile and requires immediate attention.
+**Important Note:** This analysis is based solely on a single frame of video. A more comprehensive assessment would require reviewing additional frames, analyzing audio (if available), and gathering contextual information about the individuals involved and the circumstances surrounding the event.  Immediate action should be taken to secure the scene, identify the individual, and determine his intentions. 
+Would you like me to elaborate on any specific aspect of this analysis or consider alternative interpretations?</t>
+        </is>
+      </c>
+      <c r="I92" s="5" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
       <c r="J92" s="3" t="inlineStr">
         <is>
-          <t>Base: 0.00s | FT Guided: 60.03s</t>
+          <t>Base: 0.00s | FT Guided: 103.10s</t>
         </is>
       </c>
       <c r="K92" s="4" t="inlineStr">
@@ -9248,17 +9785,39 @@
       </c>
       <c r="H93" s="4" t="inlineStr">
         <is>
-          <t>Error: HTTPConnectionPool(host='localhost', port=11434): Read timed out. (read timeout=60)</t>
-        </is>
-      </c>
-      <c r="I93" s="6" t="inlineStr">
-        <is>
-          <t>Low</t>
+          <t>Okay, let’s analyze this surveillance video sequence based on the provided activity class and visual evidence.
+**What is happening?**
+The video depicts a catastrophic event within a warehouse or industrial space. There's been a significant structural failure leading to widespread destruction of equipment, shelving units, and general debris. It appears to be a chaotic scene with items scattered across the floor and overhead. 
+**Which activities are visible?**
+* **Structural Collapse:** The most prominent activity is the collapse of shelving units and potentially parts of the warehouse structure itself.
+* **Debris Scattering:**  A massive amount of debris – boxes, pallets, equipment components, and other items – is being thrown around by the force of the event. 
+* **Movement (Implied):** While we don't see individuals directly, the movement of objects suggests a powerful force was at play. The Red Bull container indicates that this may have been an industrial or commercial space.
+**Is there any suspicious behaviour?**
+Based solely on this video, it’s difficult to determine if there was *intentional* suspicious behavior. However, the scale and nature of the event strongly suggest a sudden, unexpected force – most likely extreme weather (tornado). It's possible that the damage could have been caused by an external factor, but without further information, we cannot conclude this. 
+**Are there any threat indicators?**
+* **Structural Instability:** The primary threat indicator is the obvious structural failure. This indicates a potentially dangerous situation with ongoing risk of further collapse and injury.
+* **Uncontrolled Movement of Objects:** The flying debris represents a significant hazard – people could be struck by falling objects, or trapped under collapsing structures. 
+* **Scale of Damage:** The sheer volume of destruction suggests the force involved was substantial, indicating a potentially dangerous event.
+**Estimate the threat level as Low, Medium, or High.**
+**Threat Level: High**
+**Reasoning:**
+Here’s why I assess this as a high threat level:
+* **Significant Structural Damage:** The scale of the collapse is extreme and indicates a powerful force.
+* **Hazardous Debris:**  The uncontrolled movement of debris poses an immediate risk of injury to anyone still within the affected area. 
+* **Unpredictable Further Collapse:** There's a high probability that further sections of the structure could collapse, creating ongoing danger. 
+* **Potential for Casualties:** Given the widespread destruction and potential for entrapment, there is a significant risk of injuries or fatalities.
+**Important Note:** This analysis is based solely on the provided video footage and the given activity class description. A more comprehensive assessment would require additional information such as weather data, building structural reports, and potentially eyewitness accounts. 
+Would you like me to elaborate on any specific aspect of this analysis?</t>
+        </is>
+      </c>
+      <c r="I93" s="5" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
       <c r="J93" s="3" t="inlineStr">
         <is>
-          <t>Base: 0.00s | FT Guided: 60.04s</t>
+          <t>Base: 0.00s | FT Guided: 94.83s</t>
         </is>
       </c>
       <c r="K93" s="4" t="inlineStr">
@@ -9309,17 +9868,43 @@
       </c>
       <c r="H94" s="4" t="inlineStr">
         <is>
-          <t>Error: HTTPConnectionPool(host='localhost', port=11434): Read timed out. (read timeout=60)</t>
-        </is>
-      </c>
-      <c r="I94" s="6" t="inlineStr">
-        <is>
-          <t>Low</t>
+          <t>Okay, let’s analyze this surveillance scene based on the provided activity class and visual evidence.
+**What is happening?**
+A dark-colored vehicle has violently crashed through a concrete barrier and entered the median of a multi-lane highway. The impact has caused significant damage to the barrier and likely damaged the vehicle itself. Traffic flow is disrupted in both directions, with vehicles slowing down or stopping to observe the scene. 
+**Which activities are visible?**
+* **Vehicle Crash:** The primary activity is the catastrophic crash of the dark vehicle.
+* **Traffic Disruption:** Vehicles are reacting to the crash – some braking, others observing, and potentially creating a traffic backlog.
+* **Emergency Response (Potential):** While not immediately apparent in this frame, we can anticipate emergency services (police, paramedics) will be arriving at the scene shortly. 
+* **Barrier Damage:** The concrete barrier is severely damaged, indicating significant force was involved.
+**Is there any suspicious behaviour?**
+Based on just this single frame, it's difficult to determine if there’s *suspicious* behavior. However, the sudden and forceful nature of the crash immediately raises questions about the circumstances surrounding it. It could be a deliberate act or an accident. 
+**Are there any threat indicators?**
+Yes, several threat indicators are present:
+* **High-Speed Impact:** The vehicle was traveling at a significant speed before impact, suggesting potential reckless driving or impairment.
+* **Barrier Damage:**  The damage to the barrier indicates considerable force and could suggest an intentional act of vandalism or assault. 
+* **Disrupted Traffic:** A sudden crash disrupts traffic flow, creating a potential hazard for other drivers and pedestrians.
+**Estimate the threat level as Low, Medium, or High.**
+I would rate the threat level as **Medium**. 
+**Explain your reasoning:**
+Here’s why I've assessed it as medium:
+*   **Significant Damage &amp; Potential Injury:** The crash itself represents a significant safety hazard and could have resulted in serious injuries to the driver or other road users.
+*   **Uncertain Circumstances:** We don’t know *why* this happened. It could be an accident, but the force of the impact suggests something more. 
+*   **Disruption &amp; Risk:** The disruption to traffic creates a risk for other drivers and potentially pedestrians who may not see the situation.
+However, it's not a high threat level because we don’t have immediate evidence of malicious intent (like weapons or obvious signs of an attack). Further investigation is needed to determine the cause of the crash and whether there are any additional threats involved. 
+**Further Considerations (Based on the Image):**
+*   It would be beneficial to see subsequent frames to understand the vehicle's trajectory, speed before impact, and the condition of the driver.
+*   The presence of a bus nearby suggests a high-traffic area and potentially more vulnerable pedestrians. 
+Do you want me to focus on any specific aspect of this scene (e.g., analyzing the damage, potential causes of the crash, or emergency response)?</t>
+        </is>
+      </c>
+      <c r="I94" s="5" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
       <c r="J94" s="3" t="inlineStr">
         <is>
-          <t>Base: 0.00s | FT Guided: 60.02s</t>
+          <t>Base: 0.00s | FT Guided: 101.35s</t>
         </is>
       </c>
       <c r="K94" s="4" t="inlineStr">
@@ -9346,7 +9931,30 @@
       </c>
       <c r="D95" s="4" t="inlineStr">
         <is>
-          <t>Error: HTTPConnectionPool(host='localhost', port=11434): Read timed out. (read timeout=60)</t>
+          <t>Okay, let's analyze this surveillance video sequence.
+**What is happening?**
+The video shows a busy intersection with several vehicles waiting at a traffic light. It appears to be a typical suburban street scene during daylight hours. Cars are queued up on both sides of the intersection, likely waiting to turn or proceed straight through. 
+**Which activities are visible?**
+* **Vehicles Waiting:** The primary activity is vehicles patiently waiting for the green light.
+* **Traffic Flow (Limited):**  There's a slow and steady flow of traffic as cars proceed through the intersection after the light changes.
+* **Pedestrians (Potentially):** While not immediately obvious, there are sidewalks visible on either side of the street, suggesting pedestrians may be present, though they aren’t directly in the frame at this moment.
+**Is there any suspicious behaviour?**
+Based solely on this still image, it's difficult to definitively say if there is *suspicious* behavior. However, there are a few elements that warrant closer observation:
+* **Vehicle Positioning:** The silver sedan closest to the camera appears to be slightly angled towards the intersection and close to the crosswalk. This could be normal, but in a surveillance context, it raises a slight flag.
+* **Lack of Obvious Activity:** The scene is relatively calm, which itself can sometimes be unusual if there's an event occurring that isn’t immediately apparent.
+**Are there any threat indicators?**
+There are no *obvious* immediate threat indicators in this single frame. However:
+* **Potential for Misuse:**  The positioning of the silver sedan could potentially allow a driver to quickly move into the intersection if they were attempting to cause an accident or evade law enforcement. 
+* **Unidentified Objects:** There is a small, dark object (possibly a bag) visible on the hood of the silver sedan. This needs further investigation.
+**Estimate the threat level as Low, Medium, or High.**
+**Threat Level: Low - Medium**
+**Reasoning:**
+My assessment leans towards low-medium due to the following:
+* **No Immediate Violence:** There's no visible aggressive behavior, physical contact between vehicles, or any indication of imminent danger.
+* **Potential for Opportunistic Action:** The positioning of the silver sedan and the presence of an unidentified object on its hood suggest a *potential* risk if someone were to take advantage of the traffic flow. This is more about a possible vulnerability than an active threat. 
+* **Need for Further Investigation:**  This single frame provides limited context. A longer video sequence, coupled with analysis of vehicle speeds, driver behavior (if visible), and the nature of the object on the hood would be needed to refine the assessment.
+**Important Note:** This analysis is based solely on a still image. A full surveillance review would require analyzing the entire video stream for movement patterns, interactions between vehicles and pedestrians, and any other relevant details. 
+Would you like me to consider additional factors or analyze a longer segment of the video if available?</t>
         </is>
       </c>
       <c r="E95" s="4" t="inlineStr">
@@ -9368,17 +9976,33 @@
       </c>
       <c r="H95" s="4" t="inlineStr">
         <is>
-          <t>Error: HTTPConnectionPool(host='localhost', port=11434): Read timed out. (read timeout=60)</t>
-        </is>
-      </c>
-      <c r="I95" s="6" t="inlineStr">
-        <is>
-          <t>Low</t>
+          <t>Okay, let's analyze this surveillance scene based on the provided activity class and visual evidence.
+**What is happening?**
+The video shows a busy intersection with multiple vehicles stopped at the crosswalk. It appears to be a standard traffic situation where vehicles are waiting for a change in the traffic light. 
+**Which activities are visible?**
+* **Vehicle Stops:** The primary activity is numerous vehicles coming to a complete stop at the intersection, likely due to the traffic light.
+* **Waiting:** Vehicles are stationary and appear to be patiently awaiting their turn to proceed through the intersection.
+* **Traffic Flow (Potential):**  We can see some movement in the background as vehicles continue along the road leading into the intersection, suggesting a flow of traffic is present. 
+**Is there any suspicious behaviour?**
+Based solely on this single frame, there isn't immediately obvious suspicious behavior. However, it’s important to note that we are only seeing one moment in time. 
+**Are there any threat indicators?**
+* **Density of Vehicles:** The high density of vehicles at the intersection *could* be a potential indicator if something were to disrupt the flow – for example, an unexpected pedestrian crossing or a sudden obstruction. However, this is normal traffic congestion.
+* **Lack of Obvious Hazards:** There are no immediately visible hazards like debris in the road, accidents, or aggressive drivers.
+**Estimate the threat level as Low, Medium, or High.**
+**Threat Level: Low** 
+**Reasoning:**
+The scene depicts a typical, albeit busy, intersection. The activity class "Several vehicles are stopped at a busy intersection, likely waiting for a traffic light to change" accurately describes what is happening. There aren't any immediately apparent threats based on this single frame.  However, it’s crucial to remember that this is just one snapshot in time. A longer video sequence would be needed to assess the situation more thoroughly and identify potential risks or unusual behavior. 
+**Important Note:** This analysis is limited by the information provided – a single still image. A full threat assessment would require analyzing a continuous video stream, considering factors like driver behavior, pedestrian activity, and surrounding environment over time.</t>
+        </is>
+      </c>
+      <c r="I95" s="5" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
       <c r="J95" s="3" t="inlineStr">
         <is>
-          <t>Base: 60.03s | FT Guided: 60.01s</t>
+          <t>Base: 97.49s | FT Guided: 80.36s</t>
         </is>
       </c>
       <c r="K95" s="4" t="inlineStr">
@@ -9427,17 +10051,39 @@
       </c>
       <c r="H96" s="4" t="inlineStr">
         <is>
-          <t>Error: HTTPConnectionPool(host='localhost', port=11434): Read timed out. (read timeout=60)</t>
-        </is>
-      </c>
-      <c r="I96" s="6" t="inlineStr">
-        <is>
-          <t>Low</t>
+          <t>Okay, let's analyze this surveillance scene video sequence based on the provided activity class and visual evidence.
+**What is happening?**
+The video shows a busy traffic intersection with vehicles moving along roadways and pedestrian walkways. The elevated overpasses indicate a complex transportation hub, likely a highway interchange or major road junction. 
+**Which activities are visible?**
+* **Vehicle Traffic:** Cars, trucks, and possibly other vehicles are navigating the intersection, following lane markings and signals.
+* **Pedestrian Activity:** People are walking along sidewalks and potentially crossing at designated crosswalks under the overpasses.
+* **Traffic Control:** Traffic lights are clearly visible, regulating the flow of traffic. 
+* **Infrastructure:** The presence of elevated roadways, streetlights, signage, and pedestrian walkways indicates a well-developed urban environment.
+**Is there any suspicious behaviour?**
+Based solely on this single frame, it's difficult to definitively identify suspicious behavior. However, we can note the following that *could* warrant further investigation:
+* **Vehicle Positioning:** The positioning of vehicles in relation to lanes and intersections could be unusual if they are stopped erratically or blocking traffic flow.
+* **Pedestrian Movement:**  Unusual pedestrian movement patterns (e.g., lingering in one spot, crossing against the light) might raise concerns. 
+**Are there any threat indicators?**
+There aren't immediately obvious threat indicators within this single frame. However, the elevated roadways and high traffic volume could present potential risks if a collision or other incident were to occur. The presence of multiple vehicles and pedestrians increases the potential for harm.
+**Estimate the threat level as Low, Medium, or High.**
+**Threat Level: Low** 
+**Reasoning:**
+* **Limited Visual Information:** This is just one frame from a video sequence. We lack context about surrounding areas, time of day, and overall traffic patterns.
+* **Normal Traffic Activity:** The scene depicts typical traffic intersection activity – vehicles moving, pedestrians walking, and traffic signals operating. 
+* **No Obvious Threats:** There are no immediately visible signs of violence, suspicious individuals, or dangerous actions.
+**Important Note:**  A threat assessment based on a single frame is inherently limited. A full analysis would require reviewing the entire video sequence to identify patterns, anomalies, and potential risks. Further investigation would be needed to confirm if any of the observed activities are truly concerning. 
+---
+Would you like me to analyze additional frames from the video or consider specific aspects (e.g., time of day, weather conditions) to refine the assessment?</t>
+        </is>
+      </c>
+      <c r="I96" s="5" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
       <c r="J96" s="3" t="inlineStr">
         <is>
-          <t>Base: 0.00s | FT Guided: 60.01s</t>
+          <t>Base: 0.00s | FT Guided: 91.15s</t>
         </is>
       </c>
       <c r="K96" s="4" t="inlineStr">
@@ -9488,17 +10134,43 @@
       </c>
       <c r="H97" s="4" t="inlineStr">
         <is>
-          <t>Error: HTTPConnectionPool(host='localhost', port=11434): Read timed out. (read timeout=60)</t>
-        </is>
-      </c>
-      <c r="I97" s="6" t="inlineStr">
-        <is>
-          <t>Low</t>
+          <t>Okay, let’s analyze this surveillance scene based on the provided activity class and visual evidence.
+**What is happening?**
+The video shows a busy intersection with significant traffic control measures in place. The presence of numerous orange cones, signage, and flashing lights indicates that the normal flow of traffic has been disrupted. It appears to be a deliberate attempt to manage vehicles and pedestrians at this location. 
+**Which activities are visible?**
+* **Vehicular Traffic:** Cars are navigating around the cone barriers, suggesting they are attempting to use the intersection despite the restrictions.
+* **Pedestrian Activity:** Pedestrians are crossing the street at designated crosswalks, likely following instructions from the signage and traffic signals. 
+* **Traffic Control Personnel (Implied):** The cones and signage strongly suggest the presence of personnel directing or monitoring traffic flow – though we don't see them directly in this frame.
+* **Street Maintenance/Construction (Likely):**  The overall setup points to ongoing work, possibly road repairs, construction, or an event that requires temporary traffic management.
+**Is there any suspicious behaviour?**
+Based on a single frame, it’s difficult to definitively identify suspicious behavior. However, the unusual concentration of traffic control measures raises a slight flag. It's possible this is legitimate work, but without further context (e.g., time of day, surrounding area), it warrants closer observation. 
+**Are there any threat indicators?**
+* **Potential for Congestion:** The heavy use of cones and signage creates the potential for increased congestion and frustration among drivers.
+* **Risk of Accidents:**  The disrupted traffic flow increases the risk of accidents if drivers are not paying close attention or if pedestrians misjudge timing. 
+**Estimate the threat level as Low, Medium, or High.**
+**Threat Level: Low**
+**Reasoning:**
+At this moment, based solely on this single frame, the threat level is assessed as **Low**. Here’s why:
+* **No Obvious Threats Visible:** There are no immediately apparent threats like aggressive drivers, individuals behaving suspiciously, or signs of violence.
+* **Likely Legitimate Activity:** The setup strongly suggests a planned event – construction, roadwork, or an organized gathering – which is generally not inherently threatening. 
+* **Context Dependent:**  The threat level could increase significantly if we knew the time of day (e.g., rush hour), the location (e.g., near a sensitive area), or had access to additional frames showing the situation evolving over time.
+**Recommendations for Further Analysis:**
+To improve this assessment, I would need:
+*   **Additional Frames:**  A sequence of images/video to observe traffic flow and any changes in behavior.
+*   **Time Stamp:** The exact date and time of the recording.
+*   **Location Information:** Precise location details (street names, landmarks) for context. 
+*   **Event Details:** Any information about planned events or construction projects occurring nearby.
+Do you want me to elaborate on any specific aspect of this scene, such as potential risks associated with traffic congestion or the types of activities that might be taking place at this intersection?</t>
+        </is>
+      </c>
+      <c r="I97" s="5" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
       <c r="J97" s="3" t="inlineStr">
         <is>
-          <t>Base: 0.00s | FT Guided: 60.01s</t>
+          <t>Base: 0.00s | FT Guided: 117.46s</t>
         </is>
       </c>
       <c r="K97" s="4" t="inlineStr">
@@ -9547,17 +10219,37 @@
       </c>
       <c r="H98" s="4" t="inlineStr">
         <is>
-          <t>Error: HTTPConnectionPool(host='localhost', port=11434): Read timed out. (read timeout=60)</t>
-        </is>
-      </c>
-      <c r="I98" s="6" t="inlineStr">
-        <is>
-          <t>Low</t>
+          <t>Okay, let's analyze this surveillance scene video based on the provided activity class: "A rainy street scene with traffic and pedestrians under a cloudy sky."
+**What is happening?**
+The video depicts a typical urban street scene during inclement weather. It’s raining, indicated by reflections on the pavement and wet surfaces. Traffic is present – vehicles are moving along the road. Pedestrians are walking along the sidewalks. The overall impression is one of a normal, albeit slightly gloomy, city environment. 
+**Which activities are visible?**
+* **Traffic Flow:** Vehicles (cars, likely) are navigating the street.
+* **Pedestrian Movement:** People are walking on the sidewalk.
+* **Street Lighting &amp; Signage:** Streetlights and signage are present, indicating a public space.
+* **Urban Infrastructure:** The scene includes elements of urban infrastructure like sidewalks, curbs, and building facades.
+**Is there any suspicious behaviour?**
+Based solely on this single frame, it's difficult to definitively say if there is *suspicious* behavior. However, the following could warrant further investigation:
+* **Unusual Pedestrian Movement:**  If a pedestrian were lingering in an area for an extended period without apparent purpose, or exhibiting erratic movements, that would be noteworthy.
+* **Vehicle Behavior:** If a vehicle were stopped erratically, or moving slowly and suspiciously, it would raise concerns. 
+**Are there any threat indicators?**
+The video itself doesn't immediately present obvious *threat indicators*. However:
+* **Rainy Conditions:** Rain can reduce visibility for both pedestrians and drivers, potentially increasing the risk of accidents.
+* **Crowded Environment:** A crowded street scene increases the potential for a mass incident (e.g., stampede).
+**Estimate the threat level as Low, Medium, or High.**
+**Threat Level: Low** 
+**Reasoning:**
+The video shows a common urban environment during rainy weather. While there are inherent risks associated with traffic and pedestrian activity in inclement conditions, there's no immediately obvious evidence of criminal behavior, violence, or imminent danger. The scene is relatively calm and unremarkable.  It’s important to note that this assessment is based on *one* frame; a longer video sequence could reveal more concerning details. 
+**Important Note:** This analysis is limited by the single frame provided. A full review of the entire video sequence would be necessary for a more comprehensive threat assessment. Factors like camera angle, lighting changes, and movement patterns across multiple frames would significantly impact the evaluation.</t>
+        </is>
+      </c>
+      <c r="I98" s="5" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
       <c r="J98" s="3" t="inlineStr">
         <is>
-          <t>Base: 0.00s | FT Guided: 60.02s</t>
+          <t>Base: 0.00s | FT Guided: 100.59s</t>
         </is>
       </c>
       <c r="K98" s="4" t="inlineStr">
@@ -9606,17 +10298,38 @@
       </c>
       <c r="H99" s="4" t="inlineStr">
         <is>
-          <t>Error: HTTPConnectionPool(host='localhost', port=11434): Read timed out. (read timeout=60)</t>
-        </is>
-      </c>
-      <c r="I99" s="6" t="inlineStr">
-        <is>
-          <t>Low</t>
+          <t>Okay, let’s analyze this surveillance video sequence based on the provided activity class and visual observations.
+**What is happening?**
+The video depicts a busy intersection with vehicles navigating through it. The key element is that traffic lights are in operation – one lane has an orange light indicating permitted movement, while another has a yellow light, signaling imminent stopping. Vehicles are proceeding cautiously, likely awaiting the green light to continue. 
+**Which activities are visible?**
+* **Vehicle Movement:** Cars are actively driving and maneuvering through the intersection.
+* **Traffic Light Operation:** The traffic lights themselves are clearly visible and functioning with different colored signals.
+* **Pedestrian Presence (Implied):** While not directly visible in this frame, the presence of sidewalks and crosswalks suggests pedestrians are likely navigating the area as well. 
+**Is there any suspicious behaviour?**
+Based solely on this single frame, it's difficult to definitively identify suspicious behavior. However, we can observe:
+* **Vehicle Positioning:** The vehicles appear to be positioned in a way that could potentially lead to conflict if they were to proceed without proper signaling or awareness of other traffic. 
+* **Traffic Light Status:** The orange and yellow lights create a situation where drivers might be momentarily confused or make an incorrect decision if not paying close attention.
+**Are there any threat indicators?**
+There are no immediately obvious threat indicators in this single frame. However, the following could potentially escalate into a threat:
+* **Potential for Collision:** The combination of traffic light signals and vehicle movement creates a situation where a collision is possible if drivers aren't attentive. 
+* **Driver Distraction:**  The driver of the white SUV appears to be looking down, which could indicate distraction.
+**Estimate the threat level as Low, Medium, or High.**
+**Threat Level: Low**
+**Reasoning:**
+This single frame doesn’t present an immediate, high-risk situation. The primary risk is a potential collision due to traffic light confusion and driver behavior. However, this is a relatively common scenario in urban intersections. 
+* **Low Threat Justification:** There's no overt aggressive driving, weapons visible, or other indicators of imminent danger. It’s more about the *potential* for an accident rather than an active threat. 
+* **Further Investigation Needed:**  This assessment is based on a single frame. Continuous monitoring would be necessary to assess driver behavior, traffic flow, and any potential escalation of the situation.
+**Important Note:** This analysis is limited by the information available in this single frame. A more comprehensive risk assessment would require analyzing the entire video sequence, including vehicle speeds, driver actions, pedestrian movements, and overall traffic patterns.</t>
+        </is>
+      </c>
+      <c r="I99" s="5" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
       <c r="J99" s="3" t="inlineStr">
         <is>
-          <t>Base: 0.00s | FT Guided: 60.01s</t>
+          <t>Base: 0.00s | FT Guided: 105.73s</t>
         </is>
       </c>
       <c r="K99" s="4" t="inlineStr">
@@ -9643,7 +10356,30 @@
       </c>
       <c r="D100" s="4" t="inlineStr">
         <is>
-          <t>Error: HTTPConnectionPool(host='localhost', port=11434): Read timed out. (read timeout=60)</t>
+          <t>Okay, let's analyze this surveillance video sequence.
+**What is happening?**
+The video shows a relatively quiet suburban street scene. A white pickup truck is traveling down the road in the center lane. There are several other vehicles parked along the side of the road and some pedestrians can be seen walking on the sidewalk. It appears to be daytime, though the lighting isn't ideal. 
+**Which activities are visible?**
+*   **Vehicle Movement:** A single vehicle (white pickup) is actively moving down the street.
+*   **Pedestrian Activity:** People are walking along the sidewalks.
+*   **Parking:** Several vehicles are parked along the side of the road, likely residents or visitors. 
+**Is there any suspicious behaviour?**
+There isn't immediately obvious suspicious behavior. The driver of the pickup is traveling in a lane and doesn’t appear to be exhibiting erratic driving patterns. However, it's important to note that we can only see what's directly in front of the camera. 
+**Are there any threat indicators?**
+*   **Lack of Obvious Threats:** There are no immediately apparent threats like weapons, aggressive behavior, or unusual activity.
+*   **Potential for Speeding/Distraction:** It’s difficult to assess from this frame if the driver is speeding or distracted. 
+**Estimate the threat level as Low, Medium, or High.**
+**Threat Level: Low**
+**Reasoning:**
+Based on this single frame of video, there are no immediate indicators of a high-threat situation. The scene appears relatively normal for a suburban street. However, it's crucial to understand that this is just one snapshot in time. 
+*   **Limited Information:** We only have one frame. It’s possible other events are occurring outside the view of the camera.
+*   **Potential for Hidden Threats:** Surveillance footage needs to be analyzed over a longer period to identify patterns, potential risks, or unusual behavior that might indicate a threat. 
+**Recommendations for Further Analysis:**
+To get a more complete picture, I would recommend:
+1.  **Extended Video Review:** Analyze the entire video sequence to see if there are any changes in activity, vehicle movements, or pedestrian behavior over time.
+2.  **Contextual Information:** Gather information about the location (e.g., residential area, commercial zone) and any known events happening nearby that might influence the situation. 
+3. **Check for other cameras**: Are there other cameras in the vicinity that could provide a wider view of the scene?
+**Disclaimer:** *This analysis is based solely on the provided image. A comprehensive threat assessment would require a much more detailed review of the entire video sequence and additional contextual information.*</t>
         </is>
       </c>
       <c r="E100" s="4" t="inlineStr">
@@ -9665,17 +10401,35 @@
       </c>
       <c r="H100" s="4" t="inlineStr">
         <is>
-          <t>Error: HTTPConnectionPool(host='localhost', port=11434): Read timed out. (read timeout=60)</t>
-        </is>
-      </c>
-      <c r="I100" s="6" t="inlineStr">
-        <is>
-          <t>Low</t>
+          <t>Okay, let’s analyze this surveillance scene based on the provided activity class and visual evidence.
+**What is happening?**
+The video shows a white pickup truck moving along a two-lane road. It appears to be traveling in what seems like a normal manner within a residential area. The road has double yellow lines indicating separation of traffic lanes, which suggests it's likely a local street or neighborhood route rather than a major highway. 
+**Which activities are visible?**
+*   **Vehicle Movement:** The primary activity is the movement of the white pickup truck down the road.
+*   **Traffic Flow (Limited):** There’s limited traffic flow, with other vehicles present in the background, though they aren't directly interacting with the main subject. 
+*   **Residential Activity:**  We can see residential houses and greenery surrounding the road, indicating a typical suburban or neighborhood setting.
+**Is there any suspicious behaviour?**
+Based solely on this single frame, there isn’t immediately obvious suspicious behavior. The truck is traveling predictably within its lane. However, without additional context (speed, direction of travel relative to other vehicles, etc.), it's impossible to definitively rule out anything unusual. 
+**Are there any threat indicators?**
+There are no explicit threat indicators visible in this single frame. There’s no obvious indication of reckless driving, aggressive behavior, or potential danger. However, the double yellow lines suggest a potentially higher risk of sideswiping if another vehicle enters the lane unexpectedly. 
+**Estimate the threat level as Low, Medium, or High.**
+*   **Threat Level: Low**
+**Reasoning:**
+The threat level is assessed as low because:
+1.  **Normal Traffic Conditions:** The scene depicts a typical suburban road environment with limited traffic and no immediately apparent hazards.
+2.  **Predictable Vehicle Movement:** The pickup truck appears to be traveling in a standard manner, adhering to lane markings. 
+3. **Lack of Obvious Indicators**: There are no visible signs of reckless driving, aggressive behavior, or any other immediate threats.
+**Important Note:** This analysis is based on a single frame of video. A more comprehensive threat assessment would require analyzing the entire video sequence, considering factors like speed, direction, surrounding traffic, and any changes in behavior over time.</t>
+        </is>
+      </c>
+      <c r="I100" s="5" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
       <c r="J100" s="3" t="inlineStr">
         <is>
-          <t>Base: 60.03s | FT Guided: 60.04s</t>
+          <t>Base: 105.21s | FT Guided: 94.73s</t>
         </is>
       </c>
       <c r="K100" s="4" t="inlineStr">
@@ -9726,17 +10480,34 @@
       </c>
       <c r="H101" s="4" t="inlineStr">
         <is>
-          <t>Error: HTTPConnectionPool(host='localhost', port=11434): Read timed out. (read timeout=60)</t>
-        </is>
-      </c>
-      <c r="I101" s="6" t="inlineStr">
-        <is>
-          <t>Low</t>
+          <t>Okay, let’s analyze this surveillance scene based on the provided activity class and visual evidence.
+**What is happening?**
+The video shows a typical intersection with vehicles navigating through it. It appears to be a moderately busy street corner as evidenced by the presence of multiple cars. The traffic light is functioning, controlling the flow of vehicles. 
+**Which activities are visible?**
+* **Vehicle Movement:** Cars are actively driving into and out of the intersection, following the signals from the traffic light.
+* **Traffic Flow:** Vehicles are moving along the road within the intersection.
+* **Pedestrian Presence (Implied):** While not directly visible in this frame, the presence of a crosswalk suggests pedestrians likely use this intersection.
+**Is there any suspicious behaviour?**
+Based solely on this single frame, it's difficult to definitively say if there is *suspicious* behavior. However, we can observe:
+* **Vehicle Positioning:** The cars are positioned in a way that could be interpreted as potentially unsafe or erratic depending on their speed and proximity to the intersection. 
+**Are there any threat indicators?**
+There aren't immediately obvious threat indicators within this single frame. There is no visible violence, weapons, or aggressive actions. However:
+* **Traffic Density:** The high traffic density could be a potential factor if an accident were to occur. 
+**Estimate the threat level as Low, Medium, or High.**
+**Threat Level: Low**
+**Reasoning:**
+This single frame doesn't present any immediate, obvious threats. The scene is relatively normal for a busy intersection.  The traffic flow and functioning traffic light suggest a controlled environment. However, it’s important to note that this assessment is based on *one* frame of video. A longer sequence would be needed to fully assess the situation and identify potential risks. 
+**Important Note:** This analysis is limited by the information available in just one frame.  A more comprehensive threat assessment would require analyzing a continuous stream of footage, tracking vehicle movements over time, and looking for patterns or anomalies that might indicate a developing risk.</t>
+        </is>
+      </c>
+      <c r="I101" s="5" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
       <c r="J101" s="3" t="inlineStr">
         <is>
-          <t>Base: 0.00s | FT Guided: 60.02s</t>
+          <t>Base: 0.00s | FT Guided: 89.12s</t>
         </is>
       </c>
       <c r="K101" s="4" t="inlineStr">

</xml_diff>